<commit_message>
10 Momentum & Adam: write 8 homework problems; extend study tracker
math/10_*.qmd: 8 problems covering update-rule recall, momentum implementation,
zig-zag visualization, Adam implementation, bias-correction insight, Rastrigin
failure case, learning-rate robustness comparison, and Adam vs vanilla GD on
linear regression.

math/09_*.qmd: trim HW 03 to remove the 2/λ_max theoretical comparison; keep
the experimental "find η*" task.

misc/solo/: rename column headers (Teacher's note → Note, Student's question /
comment → Questions / comments); export Optimization sheet as standalone
optimization.csv; .gitignore now allows misc/solo/*.csv.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/misc/solo/study_plan.xlsx
+++ b/misc/solo/study_plan.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Teacher's note</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -502,7 +502,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Student's question / comment</t>
+          <t>Questions / comments</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Teacher's note</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Student's question / comment</t>
+          <t>Questions / comments</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>There's a clean theoretical bound (η &lt; 2/λ_max) - your number should match closely.</t>
+          <t>Experimental — just trial and error with the learning rate.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
@@ -1241,9 +1241,233 @@
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="4" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Chapter</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>https://hayktarkhanyan.github.io/python_math_ml_course/math/10_optim_momentum_first_order_algs.html</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Builds on chapter 09. Adam/RMSProp/Adagrad fix vanilla GD's two big weaknesses: zig-zagging on ill-conditioned problems, and slow convergence.</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Lecture 17 — Momentum, ADAM, RMSProp, Adagrad</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>https://youtu.be/JsSnSHZtG_o</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Practical 11 — Adam and friends in optimization</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>https://youtu.be/mGOCt9ZcWJg</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr"/>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>HW 01 — Write out the update rules</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Recall from lecture / notes, then verify against the notebook.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>HW 02 — Implement momentum from scratch</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr"/>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Builds on chapter 09 HW 02 (vanilla GD).</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>HW 03 — Momentum kills the zig-zag</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Side-by-side with chapter 09 HW 05. Visual punchline.</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>HW 04 — Implement Adam from scratch</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Most substantial implementation in the chapter. Follow the formulas exactly.</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>HW 05 — The bias correction matters</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr"/>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Quick experiment - the 'why' explanation is the key part.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>HW 06 — When does Adam fail?</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr"/>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Counter-example to 'always use Adam'.</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>HW 07 — Robustness to the learning rate</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr"/>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Adam's main practical sell. 5 LRs spanning 4 orders of magnitude.</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Momentum, Adam, and friends</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>HW 08 — Adam for linear regression</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr"/>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Builds on chapter 09 HW 07. Often surprising: Adam doesn't help on convex problems.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1252,6 +1476,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>